<commit_message>
Model tweaks and plots
</commit_message>
<xml_diff>
--- a/Input/age_comp_ref_coll_June21_2022 (version 1).xlsx
+++ b/Input/age_comp_ref_coll_June21_2022 (version 1).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ClonedRepositories\Otobots\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F42904EA-74C7-47CF-A380-E0BC1C95983E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73DCAA25-6A15-4451-9DB3-D8CE9BB2A8F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1005" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="2" r:id="rId1"/>
@@ -24,7 +24,6 @@
     <pivotCache cacheId="0" r:id="rId3"/>
     <pivotCache cacheId="1" r:id="rId4"/>
   </pivotCaches>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -42,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="54">
   <si>
     <t>Total</t>
   </si>
@@ -198,6 +197,12 @@
   </si>
   <si>
     <t>june 21 2022</t>
+  </si>
+  <si>
+    <t>RefAge</t>
+  </si>
+  <si>
+    <t>TestAge</t>
   </si>
 </sst>
 </file>
@@ -1276,6 +1281,39 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="168" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1314,39 +1352,6 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="10" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="10" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="10" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="10" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="10" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -17453,269 +17458,6 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000001000000}" name="PivotTable2" cacheId="0" autoFormatId="4107" applyNumberFormats="1" applyBorderFormats="1" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="1" applyWidthHeightFormats="1" dataCaption="Data" updatedVersion="6" minRefreshableVersion="3" asteriskTotals="1" showMultipleLabel="0" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" gridDropZones="1">
-  <location ref="CQ1:CU53" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="5">
-    <pivotField axis="axisRow" compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1">
-      <items count="52">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item x="15"/>
-        <item x="16"/>
-        <item x="17"/>
-        <item x="18"/>
-        <item x="19"/>
-        <item x="20"/>
-        <item x="21"/>
-        <item x="22"/>
-        <item x="23"/>
-        <item x="24"/>
-        <item x="25"/>
-        <item x="26"/>
-        <item x="27"/>
-        <item x="28"/>
-        <item x="29"/>
-        <item x="30"/>
-        <item x="31"/>
-        <item x="32"/>
-        <item x="33"/>
-        <item x="34"/>
-        <item x="35"/>
-        <item x="36"/>
-        <item x="37"/>
-        <item x="38"/>
-        <item x="39"/>
-        <item x="40"/>
-        <item x="41"/>
-        <item x="42"/>
-        <item x="43"/>
-        <item x="44"/>
-        <item x="45"/>
-        <item x="46"/>
-        <item x="47"/>
-        <item x="48"/>
-        <item x="49"/>
-        <item x="50"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField dataField="1" compact="0" numFmtId="165" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="52">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i>
-      <x v="14"/>
-    </i>
-    <i>
-      <x v="15"/>
-    </i>
-    <i>
-      <x v="16"/>
-    </i>
-    <i>
-      <x v="17"/>
-    </i>
-    <i>
-      <x v="18"/>
-    </i>
-    <i>
-      <x v="19"/>
-    </i>
-    <i>
-      <x v="20"/>
-    </i>
-    <i>
-      <x v="21"/>
-    </i>
-    <i>
-      <x v="22"/>
-    </i>
-    <i>
-      <x v="23"/>
-    </i>
-    <i>
-      <x v="24"/>
-    </i>
-    <i>
-      <x v="25"/>
-    </i>
-    <i>
-      <x v="26"/>
-    </i>
-    <i>
-      <x v="27"/>
-    </i>
-    <i>
-      <x v="28"/>
-    </i>
-    <i>
-      <x v="29"/>
-    </i>
-    <i>
-      <x v="30"/>
-    </i>
-    <i>
-      <x v="31"/>
-    </i>
-    <i>
-      <x v="32"/>
-    </i>
-    <i>
-      <x v="33"/>
-    </i>
-    <i>
-      <x v="34"/>
-    </i>
-    <i>
-      <x v="35"/>
-    </i>
-    <i>
-      <x v="36"/>
-    </i>
-    <i>
-      <x v="37"/>
-    </i>
-    <i>
-      <x v="38"/>
-    </i>
-    <i>
-      <x v="39"/>
-    </i>
-    <i>
-      <x v="40"/>
-    </i>
-    <i>
-      <x v="41"/>
-    </i>
-    <i>
-      <x v="42"/>
-    </i>
-    <i>
-      <x v="43"/>
-    </i>
-    <i>
-      <x v="44"/>
-    </i>
-    <i>
-      <x v="45"/>
-    </i>
-    <i>
-      <x v="46"/>
-    </i>
-    <i>
-      <x v="47"/>
-    </i>
-    <i>
-      <x v="48"/>
-    </i>
-    <i>
-      <x v="49"/>
-    </i>
-    <i>
-      <x v="50"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-    <i i="2">
-      <x v="2"/>
-    </i>
-    <i i="3">
-      <x v="3"/>
-    </i>
-  </colItems>
-  <dataFields count="4">
-    <dataField name="Average of Test Age3" fld="1" subtotal="average" baseField="0" baseItem="0"/>
-    <dataField name="StdDev of Test Age2" fld="1" subtotal="stdDev" baseField="0" baseItem="0"/>
-    <dataField name="Count of Test Age" fld="1" subtotal="count" baseField="0" baseItem="0"/>
-    <dataField name="Sum of CV(j)" fld="4" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="1">
-    <format dxfId="0">
-      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable1" cacheId="1" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Data" updatedVersion="6" minRefreshableVersion="3" asteriskTotals="1" showMultipleLabel="0" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" gridDropZones="1">
   <location ref="CQ56:EQ109" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="2">
@@ -18159,6 +17901,269 @@
     <dataField name="Count of Test Age" fld="1" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
+    <format dxfId="0">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000001000000}" name="PivotTable2" cacheId="0" autoFormatId="4107" applyNumberFormats="1" applyBorderFormats="1" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="1" applyWidthHeightFormats="1" dataCaption="Data" updatedVersion="6" minRefreshableVersion="3" asteriskTotals="1" showMultipleLabel="0" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" gridDropZones="1">
+  <location ref="CQ1:CU53" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="5">
+    <pivotField axis="axisRow" compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1">
+      <items count="52">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item x="30"/>
+        <item x="31"/>
+        <item x="32"/>
+        <item x="33"/>
+        <item x="34"/>
+        <item x="35"/>
+        <item x="36"/>
+        <item x="37"/>
+        <item x="38"/>
+        <item x="39"/>
+        <item x="40"/>
+        <item x="41"/>
+        <item x="42"/>
+        <item x="43"/>
+        <item x="44"/>
+        <item x="45"/>
+        <item x="46"/>
+        <item x="47"/>
+        <item x="48"/>
+        <item x="49"/>
+        <item x="50"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField dataField="1" compact="0" numFmtId="165" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="52">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i>
+      <x v="19"/>
+    </i>
+    <i>
+      <x v="20"/>
+    </i>
+    <i>
+      <x v="21"/>
+    </i>
+    <i>
+      <x v="22"/>
+    </i>
+    <i>
+      <x v="23"/>
+    </i>
+    <i>
+      <x v="24"/>
+    </i>
+    <i>
+      <x v="25"/>
+    </i>
+    <i>
+      <x v="26"/>
+    </i>
+    <i>
+      <x v="27"/>
+    </i>
+    <i>
+      <x v="28"/>
+    </i>
+    <i>
+      <x v="29"/>
+    </i>
+    <i>
+      <x v="30"/>
+    </i>
+    <i>
+      <x v="31"/>
+    </i>
+    <i>
+      <x v="32"/>
+    </i>
+    <i>
+      <x v="33"/>
+    </i>
+    <i>
+      <x v="34"/>
+    </i>
+    <i>
+      <x v="35"/>
+    </i>
+    <i>
+      <x v="36"/>
+    </i>
+    <i>
+      <x v="37"/>
+    </i>
+    <i>
+      <x v="38"/>
+    </i>
+    <i>
+      <x v="39"/>
+    </i>
+    <i>
+      <x v="40"/>
+    </i>
+    <i>
+      <x v="41"/>
+    </i>
+    <i>
+      <x v="42"/>
+    </i>
+    <i>
+      <x v="43"/>
+    </i>
+    <i>
+      <x v="44"/>
+    </i>
+    <i>
+      <x v="45"/>
+    </i>
+    <i>
+      <x v="46"/>
+    </i>
+    <i>
+      <x v="47"/>
+    </i>
+    <i>
+      <x v="48"/>
+    </i>
+    <i>
+      <x v="49"/>
+    </i>
+    <i>
+      <x v="50"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+    <i i="2">
+      <x v="2"/>
+    </i>
+    <i i="3">
+      <x v="3"/>
+    </i>
+  </colItems>
+  <dataFields count="4">
+    <dataField name="Average of Test Age3" fld="1" subtotal="average" baseField="0" baseItem="0"/>
+    <dataField name="StdDev of Test Age2" fld="1" subtotal="stdDev" baseField="0" baseItem="0"/>
+    <dataField name="Count of Test Age" fld="1" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField name="Sum of CV(j)" fld="4" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="1">
     <format dxfId="1">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
@@ -18536,14 +18541,14 @@
     <col min="16" max="23" width="8.7109375" style="2" customWidth="1"/>
     <col min="24" max="24" width="2.42578125" style="2" customWidth="1"/>
     <col min="25" max="25" width="8.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="26" max="27" width="4.42578125" style="2" customWidth="1"/>
+    <col min="26" max="26" width="3.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="4" style="2" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="8.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="8.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="8.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="30" max="30" width="1.85546875" style="2" customWidth="1"/>
-    <col min="31" max="31" width="6.7109375" style="2" customWidth="1"/>
-    <col min="32" max="32" width="6.140625" style="2" customWidth="1"/>
-    <col min="33" max="33" width="5.85546875" style="2" customWidth="1"/>
-    <col min="34" max="35" width="6.5703125" style="2" customWidth="1"/>
+    <col min="31" max="31" width="8" style="2" bestFit="1" customWidth="1"/>
+    <col min="32" max="34" width="7" style="2" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="6.5703125" style="2" customWidth="1"/>
     <col min="36" max="37" width="4.140625" style="2" customWidth="1"/>
     <col min="38" max="87" width="3.140625" style="2" customWidth="1"/>
     <col min="88" max="92" width="4.140625" style="2" customWidth="1"/>
@@ -18609,10 +18614,10 @@
       <c r="AG1" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="AH1" s="141" t="s">
+      <c r="AH1" s="125" t="s">
         <v>15</v>
       </c>
-      <c r="AI1" s="141"/>
+      <c r="AI1" s="125"/>
       <c r="AL1" s="2" t="s">
         <v>46</v>
       </c>
@@ -18659,10 +18664,10 @@
         <v>51</v>
       </c>
       <c r="R2" s="4"/>
-      <c r="U2" s="140" t="s">
+      <c r="U2" s="124" t="s">
         <v>29</v>
       </c>
-      <c r="V2" s="140"/>
+      <c r="V2" s="124"/>
       <c r="Y2" s="15">
         <v>1</v>
       </c>
@@ -19524,11 +19529,11 @@
         <v>4.1818181818181817</v>
       </c>
       <c r="AF5" s="122">
-        <f t="shared" si="2"/>
+        <f>CS5</f>
         <v>0.40451991747794397</v>
       </c>
       <c r="AG5" s="123">
-        <f t="shared" si="55"/>
+        <f>CONFIDENCE(0.05, AF5,Z5)</f>
         <v>0.23905160197543052</v>
       </c>
       <c r="AH5" s="123">
@@ -19768,12 +19773,12 @@
         <v>5</v>
       </c>
       <c r="B6" s="8"/>
-      <c r="C6" s="142" t="s">
+      <c r="C6" s="126" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="143"/>
-      <c r="E6" s="143"/>
-      <c r="F6" s="144"/>
+      <c r="D6" s="127"/>
+      <c r="E6" s="127"/>
+      <c r="F6" s="128"/>
       <c r="J6" s="34" t="s">
         <v>1</v>
       </c>
@@ -20054,10 +20059,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="8"/>
-      <c r="C7" s="145"/>
-      <c r="D7" s="146"/>
-      <c r="E7" s="146"/>
-      <c r="F7" s="147"/>
+      <c r="C7" s="129"/>
+      <c r="D7" s="130"/>
+      <c r="E7" s="130"/>
+      <c r="F7" s="131"/>
       <c r="J7" s="34" t="s">
         <v>42</v>
       </c>
@@ -20341,12 +20346,12 @@
         <v>7</v>
       </c>
       <c r="B8" s="8"/>
-      <c r="C8" s="137" t="s">
+      <c r="C8" s="132" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="138"/>
-      <c r="E8" s="138"/>
-      <c r="F8" s="139"/>
+      <c r="D8" s="133"/>
+      <c r="E8" s="133"/>
+      <c r="F8" s="134"/>
       <c r="J8" s="34" t="s">
         <v>40</v>
       </c>
@@ -20626,10 +20631,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="8"/>
-      <c r="C9" s="137"/>
-      <c r="D9" s="138"/>
-      <c r="E9" s="138"/>
-      <c r="F9" s="139"/>
+      <c r="C9" s="132"/>
+      <c r="D9" s="133"/>
+      <c r="E9" s="133"/>
+      <c r="F9" s="134"/>
       <c r="Y9" s="118">
         <v>8</v>
       </c>
@@ -21173,12 +21178,12 @@
         <v>10</v>
       </c>
       <c r="B11" s="8"/>
-      <c r="C11" s="137" t="s">
+      <c r="C11" s="132" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="138"/>
-      <c r="E11" s="138"/>
-      <c r="F11" s="139"/>
+      <c r="D11" s="133"/>
+      <c r="E11" s="133"/>
+      <c r="F11" s="134"/>
       <c r="Y11" s="118">
         <v>10</v>
       </c>
@@ -21448,10 +21453,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="8"/>
-      <c r="C12" s="137"/>
-      <c r="D12" s="138"/>
-      <c r="E12" s="138"/>
-      <c r="F12" s="139"/>
+      <c r="C12" s="132"/>
+      <c r="D12" s="133"/>
+      <c r="E12" s="133"/>
+      <c r="F12" s="134"/>
       <c r="Y12" s="15">
         <v>11</v>
       </c>
@@ -21720,12 +21725,12 @@
         <v>12</v>
       </c>
       <c r="B13" s="8"/>
-      <c r="C13" s="137" t="s">
+      <c r="C13" s="132" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="138"/>
-      <c r="E13" s="138"/>
-      <c r="F13" s="139"/>
+      <c r="D13" s="133"/>
+      <c r="E13" s="133"/>
+      <c r="F13" s="134"/>
       <c r="Y13" s="118">
         <v>12</v>
       </c>
@@ -21995,10 +22000,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="8"/>
-      <c r="C14" s="137"/>
-      <c r="D14" s="138"/>
-      <c r="E14" s="138"/>
-      <c r="F14" s="139"/>
+      <c r="C14" s="132"/>
+      <c r="D14" s="133"/>
+      <c r="E14" s="133"/>
+      <c r="F14" s="134"/>
       <c r="Y14" s="15">
         <v>13</v>
       </c>
@@ -22537,12 +22542,12 @@
         <v>15</v>
       </c>
       <c r="B16" s="8"/>
-      <c r="C16" s="124" t="s">
+      <c r="C16" s="135" t="s">
         <v>27</v>
       </c>
-      <c r="D16" s="125"/>
-      <c r="E16" s="125"/>
-      <c r="F16" s="126"/>
+      <c r="D16" s="136"/>
+      <c r="E16" s="136"/>
+      <c r="F16" s="137"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
@@ -22816,13 +22821,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="8"/>
-      <c r="C17" s="127" t="str">
+      <c r="C17" s="138" t="str">
         <f>HYPERLINK("http://www.nefsc.noaa.gov/fbp/age-prec/")</f>
         <v>http://www.nefsc.noaa.gov/fbp/age-prec/</v>
       </c>
-      <c r="D17" s="128"/>
-      <c r="E17" s="128"/>
-      <c r="F17" s="129"/>
+      <c r="D17" s="139"/>
+      <c r="E17" s="139"/>
+      <c r="F17" s="140"/>
       <c r="Y17" s="15">
         <v>16</v>
       </c>
@@ -23091,12 +23096,12 @@
         <v>17</v>
       </c>
       <c r="B18" s="8"/>
-      <c r="C18" s="130" t="s">
+      <c r="C18" s="141" t="s">
         <v>33</v>
       </c>
-      <c r="D18" s="131"/>
-      <c r="E18" s="131"/>
-      <c r="F18" s="132"/>
+      <c r="D18" s="142"/>
+      <c r="E18" s="142"/>
+      <c r="F18" s="143"/>
       <c r="Y18" s="15">
         <v>17</v>
       </c>
@@ -23365,10 +23370,10 @@
         <v>18</v>
       </c>
       <c r="B19" s="8"/>
-      <c r="C19" s="130"/>
-      <c r="D19" s="131"/>
-      <c r="E19" s="131"/>
-      <c r="F19" s="132"/>
+      <c r="C19" s="141"/>
+      <c r="D19" s="142"/>
+      <c r="E19" s="142"/>
+      <c r="F19" s="143"/>
       <c r="Y19" s="15">
         <v>18</v>
       </c>
@@ -23637,10 +23642,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="8"/>
-      <c r="C20" s="133"/>
-      <c r="D20" s="134"/>
-      <c r="E20" s="134"/>
-      <c r="F20" s="135"/>
+      <c r="C20" s="144"/>
+      <c r="D20" s="145"/>
+      <c r="E20" s="145"/>
+      <c r="F20" s="146"/>
       <c r="Y20" s="15">
         <v>19</v>
       </c>
@@ -24181,12 +24186,12 @@
         <v>21</v>
       </c>
       <c r="B22" s="8"/>
-      <c r="C22" s="136" t="s">
+      <c r="C22" s="147" t="s">
         <v>28</v>
       </c>
-      <c r="D22" s="136"/>
-      <c r="E22" s="136"/>
-      <c r="F22" s="136"/>
+      <c r="D22" s="147"/>
+      <c r="E22" s="147"/>
+      <c r="F22" s="147"/>
       <c r="Y22" s="15">
         <v>21</v>
       </c>
@@ -24455,10 +24460,10 @@
         <v>22</v>
       </c>
       <c r="B23" s="8"/>
-      <c r="C23" s="136"/>
-      <c r="D23" s="136"/>
-      <c r="E23" s="136"/>
-      <c r="F23" s="136"/>
+      <c r="C23" s="147"/>
+      <c r="D23" s="147"/>
+      <c r="E23" s="147"/>
+      <c r="F23" s="147"/>
       <c r="Y23" s="15">
         <v>22</v>
       </c>
@@ -24567,7 +24572,7 @@
         <v>0</v>
       </c>
       <c r="BB23" s="53">
-        <f t="shared" si="21"/>
+        <f>DH78</f>
         <v>1</v>
       </c>
       <c r="BC23" s="53">
@@ -29958,7 +29963,7 @@
         <v>1</v>
       </c>
       <c r="AC43" s="18" t="e">
-        <f t="shared" si="62"/>
+        <f>AB43/Z43</f>
         <v>#DIV/0!</v>
       </c>
       <c r="AE43" s="20">
@@ -29970,15 +29975,15 @@
         <v>0</v>
       </c>
       <c r="AG43" s="19" t="e">
-        <f t="shared" si="63"/>
+        <f>CONFIDENCE(0.05, AF43,Z43)</f>
         <v>#NUM!</v>
       </c>
       <c r="AH43" s="19" t="e">
-        <f t="shared" si="64"/>
+        <f>AE43-(CONFIDENCE(0.05, AF43,Z43))</f>
         <v>#NUM!</v>
       </c>
       <c r="AI43" s="19" t="e">
-        <f t="shared" si="65"/>
+        <f>AE43+(CONFIDENCE(0.05, AF43,Z43))</f>
         <v>#NUM!</v>
       </c>
       <c r="AK43" s="2">
@@ -30240,7 +30245,7 @@
         <v>43</v>
       </c>
       <c r="Z44" s="16">
-        <f t="shared" si="66"/>
+        <f>CT44</f>
         <v>1</v>
       </c>
       <c r="AA44" s="17">
@@ -30264,15 +30269,15 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AG44" s="19" t="e">
-        <f t="shared" si="63"/>
+        <f>CONFIDENCE(0.05, AF44,Z44)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="AH44" s="19" t="e">
-        <f t="shared" si="64"/>
+        <f>AE44-(CONFIDENCE(0.05, AF44,Z44))</f>
         <v>#DIV/0!</v>
       </c>
       <c r="AI44" s="19" t="e">
-        <f t="shared" si="65"/>
+        <f>AE44+(CONFIDENCE(0.05, AF44,Z44))</f>
         <v>#DIV/0!</v>
       </c>
       <c r="AK44" s="2">
@@ -45630,16 +45635,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="C16:F16"/>
+    <mergeCell ref="C17:F17"/>
+    <mergeCell ref="C18:F20"/>
+    <mergeCell ref="C22:F23"/>
+    <mergeCell ref="C13:F14"/>
     <mergeCell ref="U2:V2"/>
     <mergeCell ref="AH1:AI1"/>
     <mergeCell ref="C6:F7"/>
     <mergeCell ref="C8:F9"/>
     <mergeCell ref="C11:F12"/>
-    <mergeCell ref="C16:F16"/>
-    <mergeCell ref="C17:F17"/>
-    <mergeCell ref="C18:F20"/>
-    <mergeCell ref="C22:F23"/>
-    <mergeCell ref="C13:F14"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.5" right="0.53" top="0.76" bottom="0.55000000000000004" header="0.4" footer="0.5"/>
@@ -45657,9 +45662,24 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCE65A97-7A31-45C5-B0B2-D5C5FA0D270C}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="4" max="4" width="18.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>